<commit_message>
Fixed class ranks class switching and the expired boons issue
</commit_message>
<xml_diff>
--- a/resources/data-imports/Skills/skills.xlsx
+++ b/resources/data-imports/Skills/skills.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="4"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -274,6 +274,12 @@
   </si>
   <si>
     <t xml:space="preserve">Escape the pits of torment and the delusions that haunt your mind from the time you spent in captivity. Escape with the fury and rage of a thousand men.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transmuted Essence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transmute the very essence of the world, of the souls and the indivuals around you. transmute them with your tonics and tinctures into vile beasts or from sikly to healthy.</t>
   </si>
 </sst>
 </file>
@@ -378,34 +384,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -550,8 +556,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R33"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:R34"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32.99"/>
@@ -1078,9 +1084,9 @@
         <v>400</v>
       </c>
       <c r="F14" s="0" t="n">
-        <v>0.0015625</v>
-      </c>
-      <c r="H14" s="1" t="n">
+        <v>0.001563</v>
+      </c>
+      <c r="H14" s="0" t="n">
         <v>0.001875</v>
       </c>
       <c r="K14" s="0" t="n">
@@ -1818,6 +1824,41 @@
         <v>9</v>
       </c>
       <c r="R33" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="C34" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="D34" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="E34" s="0" t="n">
+        <v>999</v>
+      </c>
+      <c r="F34" s="0" t="n">
+        <v>0.00085</v>
+      </c>
+      <c r="G34" s="0" t="n">
+        <v>0.00125</v>
+      </c>
+      <c r="N34" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="P34" s="0" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="Q34" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="R34" s="0" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>